<commit_message>
Survey123: lower-case question names and explain merging into Connect's form
Connect's Feature service starter form is built on the Hydrants layer
with inspections as a repeat. Document replacing its survey and choices
sheets with ours, and lower-case question names and the pop-up link's
field: keys to match the portal's lower-cased fields.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WcX7gz835Uu2NoHiASCWjE
</commit_message>
<xml_diff>
--- a/docs/kit/survey123/HydrantInspection.xlsx
+++ b/docs/kit/survey123/HydrantInspection.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HydrantGUID</t>
+          <t>hydrantguid</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -592,7 +592,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GISID</t>
+          <t>gisid</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lat</t>
+          <t>lat</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -695,7 +695,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lon</t>
+          <t>lon</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -782,7 +782,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>InspDate</t>
+          <t>inspdate</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EngineCo</t>
+          <t>engineco</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>inspector</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -880,7 +880,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>EngineCo=${EngineCo} or name='Other'</t>
+          <t>engineco=${engineco} or name='Other'</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FoundAtLoc</t>
+          <t>foundatloc</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -975,7 +975,7 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>${FoundAtLoc} = 'Yes'</t>
+          <t>${foundatloc} = 'Yes'</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Operable</t>
+          <t>operable</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Corrosion</t>
+          <t>corrosion</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gauge</t>
+          <t>gauge</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Spindle</t>
+          <t>spindle</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>LowPressure</t>
+          <t>lowpressure</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1171,7 +1171,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>if(string-length(${Gauge}) &gt; 0 and string-length(${Spindle}) &gt; 0 and number(${Gauge}) &lt; number(${Spindle}), 'Yes', 'No')</t>
+          <t>if(string-length(${gauge}) &gt; 0 and string-length(${spindle}) &gt; 0 and number(${gauge}) &lt; number(${spindle}), 'Yes', 'No')</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CapsMissing</t>
+          <t>capsmissing</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ShutoffValve</t>
+          <t>shutoffvalve</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Obstructed</t>
+          <t>obstructed</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MissSerial</t>
+          <t>missserial</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MissSpindle</t>
+          <t>missspindle</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MissMainSize</t>
+          <t>missmainsize</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MissShutoffDist</t>
+          <t>missshutoffdist</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DmgThreads</t>
+          <t>dmgthreads</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>StrippedSpindle</t>
+          <t>strippedspindle</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Leak</t>
+          <t>leak</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PaintedOver</t>
+          <t>paintedover</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DmgCap</t>
+          <t>dmgcap</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HardToOperate</t>
+          <t>hardtooperate</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NeedsFollowup</t>
+          <t>needsfollowup</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1780,7 +1780,7 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>if(${FoundAtLoc} = 'No' or ${Operable} != 'Yes' or ${LowPressure} = 'Yes' or number(${CapsMissing}) &gt; 0 or (string-length(${ShutoffValve}) &gt; 0 and ${ShutoffValve} != 'OK') or ${Obstructed} = 'Yes' or count-selected(${markings}) &gt; 0 or count-selected(${issues}) &gt; 0, 'Yes', 'No')</t>
+          <t>if(${foundatloc} = 'No' or ${operable} != 'Yes' or ${lowpressure} = 'Yes' or number(${capsmissing}) &gt; 0 or (string-length(${shutoffvalve}) &gt; 0 and ${shutoffvalve} != 'OK') or ${obstructed} = 'Yes' or count-selected(${markings}) &gt; 0 or count-selected(${issues}) &gt; 0, 'Yes', 'No')</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
@@ -1802,7 +1802,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>remarks</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>${NeedsFollowup} = 'Yes'</t>
+          <t>${needsfollowup} = 'Yes'</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>EngineCo</t>
+          <t>engineco</t>
         </is>
       </c>
     </row>
@@ -14148,7 +14148,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>concat(${GISID}, ' ', format-date(${InspDate}, '%Y-%m-%d'))</t>
+          <t>concat(${gisid}, ' ', format-date(${inspdate}, '%Y-%m-%d'))</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>

</xml_diff>